<commit_message>
3.1.0: Added ODH Usual Work support sample
</commit_message>
<xml_diff>
--- a/src/resources/Fhir_Cohort_Import_Template.xlsx
+++ b/src/resources/Fhir_Cohort_Import_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mriley7/workspace/FHIRSheets/src/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{519438E7-7F8B-7846-8159-A74603AF77C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CAA3F64-7645-7244-B76F-1FB4FCBFC7C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18020" firstSheet="1" activeTab="4" xr2:uid="{B7CAF98F-F4CF-4673-A736-BDE9BA8D985C}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17940" firstSheet="1" activeTab="4" xr2:uid="{B7CAF98F-F4CF-4673-A736-BDE9BA8D985C}"/>
   </bookViews>
   <sheets>
     <sheet name="How To Use This Workbook" sheetId="6" r:id="rId1"/>
@@ -111,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="419">
   <si>
     <t>How To Use This Workbook</t>
   </si>
@@ -1371,6 +1371,48 @@
   </si>
   <si>
     <t>Provider's Telecom System</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>ODH Usual Work Category</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/us/odh/StructureDefinition/odh-UsualWork</t>
+  </si>
+  <si>
+    <t>coding</t>
+  </si>
+  <si>
+    <t>ODH Ususal Work Code</t>
+  </si>
+  <si>
+    <t>http://loinc.org^21843-8^History of Usual occupation</t>
+  </si>
+  <si>
+    <t>ODH Usual Work Industry</t>
+  </si>
+  <si>
+    <t>Observation.component[code=21844-6].valueCodeableConcept</t>
+  </si>
+  <si>
+    <t>ODH Usual Work Occupation</t>
+  </si>
+  <si>
+    <t>http://terminology.hl7.org/CodeSystem/observation-category^social-history</t>
+  </si>
+  <si>
+    <t>Observation.period.start</t>
+  </si>
+  <si>
+    <t>Observation.period.end</t>
+  </si>
+  <si>
+    <t>ODH Usual Work Start Date</t>
+  </si>
+  <si>
+    <t>ODH Usual Work End Date</t>
   </si>
 </sst>
 </file>
@@ -1964,7 +2006,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="28" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="29" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2263,24 +2305,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="4" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -2290,6 +2332,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="3" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Explanatory Text" xfId="2" builtinId="53"/>
@@ -2303,11 +2346,11 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFFF8A1"/>
       <color rgb="FFFFA1A1"/>
       <color rgb="FFA1FFEF"/>
       <color rgb="FFA1FFAC"/>
       <color rgb="FFD9FFA1"/>
-      <color rgb="FFFFF8A1"/>
       <color rgb="FFFFCEA1"/>
       <color rgb="FFFFA1D9"/>
       <color rgb="FFD9A1FF"/>
@@ -2709,36 +2752,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="20" x14ac:dyDescent="0.2">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="125" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="127"/>
+      <c r="B1" s="125"/>
     </row>
     <row r="2" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="124" t="s">
+      <c r="A2" s="123" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="124"/>
-      <c r="C2" s="124"/>
+      <c r="B2" s="123"/>
+      <c r="C2" s="123"/>
     </row>
     <row r="3" spans="1:3" ht="103.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="126" t="s">
+      <c r="A3" s="124" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="126"/>
+      <c r="B3" s="124"/>
     </row>
     <row r="4" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="125" t="s">
+      <c r="A4" s="122" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="125"/>
-      <c r="C4" s="125"/>
+      <c r="B4" s="122"/>
+      <c r="C4" s="122"/>
     </row>
     <row r="5" spans="1:3" ht="40.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="123" t="s">
+      <c r="A5" s="127" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="123"/>
+      <c r="B5" s="127"/>
     </row>
     <row r="6" spans="1:3" ht="64" x14ac:dyDescent="0.2">
       <c r="A6" s="97" t="s">
@@ -2773,35 +2816,35 @@
       </c>
     </row>
     <row r="10" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="124" t="s">
+      <c r="A10" s="123" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="124"/>
-      <c r="C10" s="124"/>
+      <c r="B10" s="123"/>
+      <c r="C10" s="123"/>
     </row>
     <row r="11" spans="1:3" ht="37.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="126" t="s">
+      <c r="A11" s="124" t="s">
         <v>300</v>
       </c>
-      <c r="B11" s="126"/>
+      <c r="B11" s="124"/>
     </row>
     <row r="12" spans="1:3" ht="37.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="122" t="s">
+      <c r="A12" s="126" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="122"/>
+      <c r="B12" s="126"/>
     </row>
     <row r="13" spans="1:3" ht="37.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="122" t="s">
+      <c r="A13" s="126" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="122"/>
+      <c r="B13" s="126"/>
     </row>
     <row r="14" spans="1:3" ht="37.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="122" t="s">
+      <c r="A14" s="126" t="s">
         <v>303</v>
       </c>
-      <c r="B14" s="122"/>
+      <c r="B14" s="126"/>
     </row>
     <row r="15" spans="1:3" ht="36" x14ac:dyDescent="0.2">
       <c r="A15" s="98" t="s">
@@ -2858,16 +2901,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A10:C10"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A10:C10"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A6" location="ResourceDefinitions!A1" display="ResourceDefinitions" xr:uid="{21E4973D-DCF1-4F08-A5DE-B12BC88A3D35}"/>
@@ -4159,7 +4202,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D010D53-A2B8-4D7D-8239-2883E618B035}">
-  <dimension ref="A1:EC16"/>
+  <dimension ref="A1:EI16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="30" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.6640625" customWidth="1"/>
@@ -4173,7 +4216,7 @@
     <col min="103" max="103" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:133" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:139" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="25" t="s">
         <v>31</v>
       </c>
@@ -4307,12 +4350,22 @@
       <c r="DW1" s="91"/>
       <c r="DX1" s="91"/>
       <c r="DY1" s="91"/>
-      <c r="DZ1" s="81"/>
+      <c r="DZ1" s="81" t="s">
+        <v>405</v>
+      </c>
       <c r="EA1" s="81"/>
       <c r="EB1" s="81"/>
       <c r="EC1" s="81"/>
-    </row>
-    <row r="2" spans="1:133" s="2" customFormat="1" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="ED1" s="82" t="s">
+        <v>405</v>
+      </c>
+      <c r="EE1" s="82"/>
+      <c r="EF1" s="82"/>
+      <c r="EG1" s="82"/>
+      <c r="EH1" s="82"/>
+      <c r="EI1" s="82"/>
+    </row>
+    <row r="2" spans="1:139" s="2" customFormat="1" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="29" t="s">
         <v>33</v>
       </c>
@@ -4712,8 +4765,26 @@
       <c r="EC2" s="60" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="3" spans="1:133" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="ED2" s="62" t="s">
+        <v>315</v>
+      </c>
+      <c r="EE2" s="62" t="s">
+        <v>102</v>
+      </c>
+      <c r="EF2" s="62" t="s">
+        <v>412</v>
+      </c>
+      <c r="EG2" s="62" t="s">
+        <v>97</v>
+      </c>
+      <c r="EH2" s="62" t="s">
+        <v>415</v>
+      </c>
+      <c r="EI2" s="62" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="3" spans="1:139" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="31" t="s">
         <v>35</v>
       </c>
@@ -4924,7 +4995,7 @@
         <v>16</v>
       </c>
       <c r="BT3" s="56" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="BU3" s="56" t="s">
         <v>141</v>
@@ -5109,8 +5180,26 @@
       <c r="EC3" s="60" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="4" spans="1:133" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="ED3" s="62" t="s">
+        <v>408</v>
+      </c>
+      <c r="EE3" s="62" t="s">
+        <v>134</v>
+      </c>
+      <c r="EF3" s="62" t="s">
+        <v>16</v>
+      </c>
+      <c r="EG3" s="62" t="s">
+        <v>16</v>
+      </c>
+      <c r="EH3" s="62" t="s">
+        <v>139</v>
+      </c>
+      <c r="EI3" s="62" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="4" spans="1:139" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="32" t="s">
         <v>37</v>
       </c>
@@ -5332,8 +5421,14 @@
       <c r="EA4" s="61"/>
       <c r="EB4" s="61"/>
       <c r="EC4" s="60"/>
-    </row>
-    <row r="5" spans="1:133" ht="65.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="ED4" s="63"/>
+      <c r="EE4" s="63"/>
+      <c r="EF4" s="63"/>
+      <c r="EG4" s="62"/>
+      <c r="EH4" s="62"/>
+      <c r="EI4" s="62"/>
+    </row>
+    <row r="5" spans="1:139" ht="65.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="27" t="s">
         <v>39</v>
       </c>
@@ -5727,8 +5822,26 @@
       <c r="EC5" s="61" t="s">
         <v>388</v>
       </c>
-    </row>
-    <row r="6" spans="1:133" s="2" customFormat="1" ht="52.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="ED5" s="63" t="s">
+        <v>407</v>
+      </c>
+      <c r="EE5" s="63" t="s">
+        <v>407</v>
+      </c>
+      <c r="EF5" s="63" t="s">
+        <v>407</v>
+      </c>
+      <c r="EG5" s="63" t="s">
+        <v>407</v>
+      </c>
+      <c r="EH5" s="63" t="s">
+        <v>407</v>
+      </c>
+      <c r="EI5" s="63" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="6" spans="1:139" s="2" customFormat="1" ht="52.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="34" t="s">
         <v>41</v>
       </c>
@@ -6126,8 +6239,26 @@
       <c r="EC6" s="89" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="7" spans="1:133" ht="16" x14ac:dyDescent="0.2">
+      <c r="ED6" s="89" t="s">
+        <v>406</v>
+      </c>
+      <c r="EE6" s="89" t="s">
+        <v>409</v>
+      </c>
+      <c r="EF6" s="89" t="s">
+        <v>411</v>
+      </c>
+      <c r="EG6" s="89" t="s">
+        <v>413</v>
+      </c>
+      <c r="EH6" s="89" t="s">
+        <v>417</v>
+      </c>
+      <c r="EI6" s="89" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="7" spans="1:139" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="119"/>
       <c r="B7" s="5"/>
       <c r="C7" s="16"/>
@@ -6263,8 +6394,18 @@
       <c r="EA7" s="17"/>
       <c r="EB7" s="17"/>
       <c r="EC7" s="17"/>
-    </row>
-    <row r="8" spans="1:133" x14ac:dyDescent="0.2">
+      <c r="ED7" s="131" t="s">
+        <v>414</v>
+      </c>
+      <c r="EE7" s="17" t="s">
+        <v>410</v>
+      </c>
+      <c r="EF7" s="17"/>
+      <c r="EG7" s="17"/>
+      <c r="EH7" s="17"/>
+      <c r="EI7" s="17"/>
+    </row>
+    <row r="8" spans="1:139" x14ac:dyDescent="0.2">
       <c r="A8" s="120"/>
       <c r="B8" s="5"/>
       <c r="C8" s="20"/>
@@ -6286,7 +6427,7 @@
       <c r="DB8" s="8"/>
       <c r="DY8" s="21"/>
     </row>
-    <row r="9" spans="1:133" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:139" x14ac:dyDescent="0.2">
       <c r="A9" s="120"/>
       <c r="B9" s="5"/>
       <c r="C9" s="20"/>
@@ -6308,7 +6449,7 @@
       <c r="DB9" s="8"/>
       <c r="DY9" s="21"/>
     </row>
-    <row r="10" spans="1:133" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:139" x14ac:dyDescent="0.2">
       <c r="A10" s="120"/>
       <c r="B10" s="5"/>
       <c r="C10" s="20"/>
@@ -6330,7 +6471,7 @@
       <c r="DB10" s="8"/>
       <c r="DY10" s="21"/>
     </row>
-    <row r="11" spans="1:133" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:139" x14ac:dyDescent="0.2">
       <c r="A11" s="120"/>
       <c r="B11" s="5"/>
       <c r="C11" s="20"/>
@@ -6352,7 +6493,7 @@
       <c r="DB11" s="8"/>
       <c r="DY11" s="21"/>
     </row>
-    <row r="12" spans="1:133" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:139" x14ac:dyDescent="0.2">
       <c r="A12" s="120"/>
       <c r="B12" s="5"/>
       <c r="C12" s="20"/>
@@ -6374,7 +6515,7 @@
       <c r="DB12" s="8"/>
       <c r="DY12" s="21"/>
     </row>
-    <row r="13" spans="1:133" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:139" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="120"/>
       <c r="B13" s="5"/>
       <c r="C13" s="20"/>
@@ -6396,7 +6537,7 @@
       <c r="DB13" s="8"/>
       <c r="DY13" s="21"/>
     </row>
-    <row r="14" spans="1:133" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:139" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="120"/>
       <c r="B14" s="5"/>
       <c r="C14" s="20"/>
@@ -6418,7 +6559,7 @@
       <c r="DB14" s="8"/>
       <c r="DY14" s="21"/>
     </row>
-    <row r="15" spans="1:133" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:139" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="120"/>
       <c r="B15" s="5"/>
       <c r="C15" s="20"/>
@@ -6440,7 +6581,7 @@
       <c r="DB15" s="8"/>
       <c r="DY15" s="21"/>
     </row>
-    <row r="16" spans="1:133" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:139" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="121"/>
       <c r="B16" s="6"/>
       <c r="C16" s="9"/>
@@ -6574,6 +6715,12 @@
       <c r="EA16" s="10"/>
       <c r="EB16" s="10"/>
       <c r="EC16" s="10"/>
+      <c r="ED16" s="10"/>
+      <c r="EE16" s="10"/>
+      <c r="EF16" s="10"/>
+      <c r="EG16" s="10"/>
+      <c r="EH16" s="10"/>
+      <c r="EI16" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6645,6 +6792,12 @@
     <hyperlink ref="EA5:EC5" r:id="rId63" display="http://hl7.org/fhir/us/core/StructureDefinition/us-core-servicerequest" xr:uid="{E0BF5631-D2C1-4A47-9C6E-09B7D0F51C95}"/>
     <hyperlink ref="DL5" r:id="rId64" xr:uid="{849A955B-0D4E-8442-8CA3-3E2505A237A3}"/>
     <hyperlink ref="DM5" r:id="rId65" xr:uid="{B9C03468-74AD-8545-941B-B6346D33A378}"/>
+    <hyperlink ref="ED5" r:id="rId66" xr:uid="{058ADC11-D76F-8A44-8FF2-CF1DD58657F4}"/>
+    <hyperlink ref="ED7" r:id="rId67" xr:uid="{76B4A4C3-F620-294F-B07F-36E44435B509}"/>
+    <hyperlink ref="EE5:EG5" r:id="rId68" display="http://hl7.org/fhir/us/odh/StructureDefinition/odh-UsualWork" xr:uid="{C1DC378C-A920-C94C-86AB-5AD8AFAF335C}"/>
+    <hyperlink ref="EE5" r:id="rId69" xr:uid="{90A04B1B-2387-7145-B4C5-65AEBF36B6BF}"/>
+    <hyperlink ref="EH5" r:id="rId70" xr:uid="{5F45FC77-8D58-F344-8C34-34B11582A41D}"/>
+    <hyperlink ref="EI5" r:id="rId71" xr:uid="{EFDDC6B3-5206-AB4B-8367-206AC1B29EA0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
3.1.2: Added pregnancy status as a directly supported resource in the main fhir sheet
</commit_message>
<xml_diff>
--- a/src/resources/Fhir_Cohort_Import_Template.xlsx
+++ b/src/resources/Fhir_Cohort_Import_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mriley7/workspace/FHIRSheets/src/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CAA3F64-7645-7244-B76F-1FB4FCBFC7C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A5E55B-EBA1-C04C-83F5-2BFC8801C26C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17940" firstSheet="1" activeTab="4" xr2:uid="{B7CAF98F-F4CF-4673-A736-BDE9BA8D985C}"/>
+    <workbookView xWindow="-38400" yWindow="-1360" windowWidth="38400" windowHeight="21000" firstSheet="1" activeTab="4" xr2:uid="{B7CAF98F-F4CF-4673-A736-BDE9BA8D985C}"/>
   </bookViews>
   <sheets>
     <sheet name="How To Use This Workbook" sheetId="6" r:id="rId1"/>
@@ -111,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="419">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1101" uniqueCount="426">
   <si>
     <t>How To Use This Workbook</t>
   </si>
@@ -1413,6 +1413,27 @@
   </si>
   <si>
     <t>ODH Usual Work End Date</t>
+  </si>
+  <si>
+    <t>Pregnancy status</t>
+  </si>
+  <si>
+    <t>Pregnancy Code</t>
+  </si>
+  <si>
+    <t>http://loinc.org^82810-3</t>
+  </si>
+  <si>
+    <t>Pregnancy Category</t>
+  </si>
+  <si>
+    <t>Pregnancy Status time issued</t>
+  </si>
+  <si>
+    <t>Pregnancy Status Effective Date</t>
+  </si>
+  <si>
+    <t>Pregnancy Status Value</t>
   </si>
 </sst>
 </file>
@@ -2346,11 +2367,11 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFD9FFA1"/>
       <color rgb="FFFFF8A1"/>
       <color rgb="FFFFA1A1"/>
       <color rgb="FFA1FFEF"/>
       <color rgb="FFA1FFAC"/>
-      <color rgb="FFD9FFA1"/>
       <color rgb="FFFFCEA1"/>
       <color rgb="FFFFA1D9"/>
       <color rgb="FFD9A1FF"/>
@@ -4202,7 +4223,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D010D53-A2B8-4D7D-8239-2883E618B035}">
-  <dimension ref="A1:EI16"/>
+  <dimension ref="A1:EO16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="30" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.6640625" customWidth="1"/>
@@ -4216,7 +4237,7 @@
     <col min="103" max="103" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:139" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:145" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="25" t="s">
         <v>31</v>
       </c>
@@ -4364,8 +4385,14 @@
       <c r="EG1" s="82"/>
       <c r="EH1" s="82"/>
       <c r="EI1" s="82"/>
+      <c r="EJ1" s="65"/>
+      <c r="EK1" s="65"/>
+      <c r="EL1" s="65"/>
+      <c r="EM1" s="65"/>
+      <c r="EN1" s="65"/>
+      <c r="EO1" s="65"/>
     </row>
-    <row r="2" spans="1:139" s="2" customFormat="1" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:145" s="2" customFormat="1" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="29" t="s">
         <v>33</v>
       </c>
@@ -4783,8 +4810,26 @@
       <c r="EI2" s="62" t="s">
         <v>416</v>
       </c>
+      <c r="EJ2" s="64" t="s">
+        <v>95</v>
+      </c>
+      <c r="EK2" s="64" t="s">
+        <v>102</v>
+      </c>
+      <c r="EL2" s="64" t="s">
+        <v>315</v>
+      </c>
+      <c r="EM2" s="64" t="s">
+        <v>96</v>
+      </c>
+      <c r="EN2" s="64" t="s">
+        <v>103</v>
+      </c>
+      <c r="EO2" s="64" t="s">
+        <v>97</v>
+      </c>
     </row>
-    <row r="3" spans="1:139" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:145" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="31" t="s">
         <v>35</v>
       </c>
@@ -5198,8 +5243,26 @@
       <c r="EI3" s="62" t="s">
         <v>139</v>
       </c>
+      <c r="EJ3" s="64" t="s">
+        <v>134</v>
+      </c>
+      <c r="EK3" s="64" t="s">
+        <v>16</v>
+      </c>
+      <c r="EL3" s="64" t="s">
+        <v>18</v>
+      </c>
+      <c r="EM3" s="64" t="s">
+        <v>141</v>
+      </c>
+      <c r="EN3" s="64" t="s">
+        <v>139</v>
+      </c>
+      <c r="EO3" s="64" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="4" spans="1:139" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:145" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="32" t="s">
         <v>37</v>
       </c>
@@ -5427,8 +5490,22 @@
       <c r="EG4" s="62"/>
       <c r="EH4" s="62"/>
       <c r="EI4" s="62"/>
+      <c r="EJ4" s="65" t="s">
+        <v>172</v>
+      </c>
+      <c r="EK4" s="65" t="s">
+        <v>177</v>
+      </c>
+      <c r="EL4" s="65" t="s">
+        <v>320</v>
+      </c>
+      <c r="EM4" s="65"/>
+      <c r="EN4" s="65"/>
+      <c r="EO4" s="65" t="s">
+        <v>173</v>
+      </c>
     </row>
-    <row r="5" spans="1:139" ht="65.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:145" ht="65.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="27" t="s">
         <v>39</v>
       </c>
@@ -5840,8 +5917,26 @@
       <c r="EI5" s="63" t="s">
         <v>407</v>
       </c>
+      <c r="EJ5" s="64" t="s">
+        <v>195</v>
+      </c>
+      <c r="EK5" s="64" t="s">
+        <v>195</v>
+      </c>
+      <c r="EL5" s="65" t="s">
+        <v>195</v>
+      </c>
+      <c r="EM5" s="64" t="s">
+        <v>195</v>
+      </c>
+      <c r="EN5" s="64" t="s">
+        <v>195</v>
+      </c>
+      <c r="EO5" s="64" t="s">
+        <v>195</v>
+      </c>
     </row>
-    <row r="6" spans="1:139" s="2" customFormat="1" ht="52.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:145" s="2" customFormat="1" ht="52.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="34" t="s">
         <v>41</v>
       </c>
@@ -6257,8 +6352,26 @@
       <c r="EI6" s="89" t="s">
         <v>418</v>
       </c>
+      <c r="EJ6" s="89" t="s">
+        <v>419</v>
+      </c>
+      <c r="EK6" s="89" t="s">
+        <v>420</v>
+      </c>
+      <c r="EL6" s="89" t="s">
+        <v>422</v>
+      </c>
+      <c r="EM6" s="89" t="s">
+        <v>423</v>
+      </c>
+      <c r="EN6" s="89" t="s">
+        <v>424</v>
+      </c>
+      <c r="EO6" s="89" t="s">
+        <v>425</v>
+      </c>
     </row>
-    <row r="7" spans="1:139" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:145" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="119"/>
       <c r="B7" s="5"/>
       <c r="C7" s="16"/>
@@ -6404,8 +6517,18 @@
       <c r="EG7" s="17"/>
       <c r="EH7" s="17"/>
       <c r="EI7" s="17"/>
+      <c r="EJ7" s="17"/>
+      <c r="EK7" t="s">
+        <v>421</v>
+      </c>
+      <c r="EL7" s="131" t="s">
+        <v>414</v>
+      </c>
+      <c r="EM7" s="17"/>
+      <c r="EN7" s="17"/>
+      <c r="EO7" s="17"/>
     </row>
-    <row r="8" spans="1:139" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:145" x14ac:dyDescent="0.2">
       <c r="A8" s="120"/>
       <c r="B8" s="5"/>
       <c r="C8" s="20"/>
@@ -6427,7 +6550,7 @@
       <c r="DB8" s="8"/>
       <c r="DY8" s="21"/>
     </row>
-    <row r="9" spans="1:139" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:145" x14ac:dyDescent="0.2">
       <c r="A9" s="120"/>
       <c r="B9" s="5"/>
       <c r="C9" s="20"/>
@@ -6449,7 +6572,7 @@
       <c r="DB9" s="8"/>
       <c r="DY9" s="21"/>
     </row>
-    <row r="10" spans="1:139" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:145" x14ac:dyDescent="0.2">
       <c r="A10" s="120"/>
       <c r="B10" s="5"/>
       <c r="C10" s="20"/>
@@ -6471,7 +6594,7 @@
       <c r="DB10" s="8"/>
       <c r="DY10" s="21"/>
     </row>
-    <row r="11" spans="1:139" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:145" x14ac:dyDescent="0.2">
       <c r="A11" s="120"/>
       <c r="B11" s="5"/>
       <c r="C11" s="20"/>
@@ -6493,7 +6616,7 @@
       <c r="DB11" s="8"/>
       <c r="DY11" s="21"/>
     </row>
-    <row r="12" spans="1:139" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:145" x14ac:dyDescent="0.2">
       <c r="A12" s="120"/>
       <c r="B12" s="5"/>
       <c r="C12" s="20"/>
@@ -6515,7 +6638,7 @@
       <c r="DB12" s="8"/>
       <c r="DY12" s="21"/>
     </row>
-    <row r="13" spans="1:139" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:145" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="120"/>
       <c r="B13" s="5"/>
       <c r="C13" s="20"/>
@@ -6537,7 +6660,7 @@
       <c r="DB13" s="8"/>
       <c r="DY13" s="21"/>
     </row>
-    <row r="14" spans="1:139" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:145" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="120"/>
       <c r="B14" s="5"/>
       <c r="C14" s="20"/>
@@ -6559,7 +6682,7 @@
       <c r="DB14" s="8"/>
       <c r="DY14" s="21"/>
     </row>
-    <row r="15" spans="1:139" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:145" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="120"/>
       <c r="B15" s="5"/>
       <c r="C15" s="20"/>
@@ -6581,7 +6704,7 @@
       <c r="DB15" s="8"/>
       <c r="DY15" s="21"/>
     </row>
-    <row r="16" spans="1:139" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:145" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="121"/>
       <c r="B16" s="6"/>
       <c r="C16" s="9"/>
@@ -6721,6 +6844,12 @@
       <c r="EG16" s="10"/>
       <c r="EH16" s="10"/>
       <c r="EI16" s="10"/>
+      <c r="EJ16" s="10"/>
+      <c r="EK16" s="10"/>
+      <c r="EL16" s="10"/>
+      <c r="EM16" s="10"/>
+      <c r="EN16" s="10"/>
+      <c r="EO16" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6798,6 +6927,16 @@
     <hyperlink ref="EE5" r:id="rId69" xr:uid="{90A04B1B-2387-7145-B4C5-65AEBF36B6BF}"/>
     <hyperlink ref="EH5" r:id="rId70" xr:uid="{5F45FC77-8D58-F344-8C34-34B11582A41D}"/>
     <hyperlink ref="EI5" r:id="rId71" xr:uid="{EFDDC6B3-5206-AB4B-8367-206AC1B29EA0}"/>
+    <hyperlink ref="EK5" r:id="rId72" xr:uid="{98BF0F1D-F44E-A544-BD9A-819A1F0775F2}"/>
+    <hyperlink ref="EK4" r:id="rId73" xr:uid="{65C1B558-168A-4F4E-A855-16D87796C211}"/>
+    <hyperlink ref="EO4" r:id="rId74" xr:uid="{EB56323F-1B2E-CA4A-841D-8D20DC90800B}"/>
+    <hyperlink ref="EJ4" r:id="rId75" xr:uid="{B59DC2D6-2E40-7440-8BDB-4E6120670694}"/>
+    <hyperlink ref="EO5" r:id="rId76" xr:uid="{1BB9C402-2A9C-1040-BF9B-0D22FCF407E0}"/>
+    <hyperlink ref="EM5" r:id="rId77" xr:uid="{BE80C563-B20B-0A40-BEBF-347FB731295B}"/>
+    <hyperlink ref="EJ5" r:id="rId78" xr:uid="{43C1F3F8-A3CE-904F-8AA8-D9D9C3DF991D}"/>
+    <hyperlink ref="EL5" r:id="rId79" xr:uid="{CDD43975-5BD5-064D-8BCC-0199351FAE79}"/>
+    <hyperlink ref="EN5" r:id="rId80" xr:uid="{1EC99C06-4DFA-5744-B2FD-EF6D5335B91B}"/>
+    <hyperlink ref="EL7" r:id="rId81" xr:uid="{CDED130F-8B5B-9C48-B37B-54A9359AE8D2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
3.1.3: Fixed issue with us-core-pregnancy status url. Fixed some naming conventions within the Reference Sheet
</commit_message>
<xml_diff>
--- a/src/resources/Fhir_Cohort_Import_Template.xlsx
+++ b/src/resources/Fhir_Cohort_Import_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mriley7/workspace/FHIRSheets/src/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A5E55B-EBA1-C04C-83F5-2BFC8801C26C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCBA98F9-27E5-D246-8304-92109B1EBBA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="-1360" windowWidth="38400" windowHeight="21000" firstSheet="1" activeTab="4" xr2:uid="{B7CAF98F-F4CF-4673-A736-BDE9BA8D985C}"/>
+    <workbookView xWindow="-38400" yWindow="-1360" windowWidth="38400" windowHeight="21000" xr2:uid="{B7CAF98F-F4CF-4673-A736-BDE9BA8D985C}"/>
   </bookViews>
   <sheets>
     <sheet name="How To Use This Workbook" sheetId="6" r:id="rId1"/>
@@ -111,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1101" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1136" uniqueCount="445">
   <si>
     <t>How To Use This Workbook</t>
   </si>
@@ -1316,9 +1316,6 @@
     <t>http://hl7.org/fhir/us/core/StructureDefinition/us-core-condition-problems-health-concerns</t>
   </si>
   <si>
-    <t>Smoking Status Effective Date</t>
-  </si>
-  <si>
     <t>PractitionerRole.code.[0]</t>
   </si>
   <si>
@@ -1427,13 +1424,73 @@
     <t>Pregnancy Category</t>
   </si>
   <si>
-    <t>Pregnancy Status time issued</t>
-  </si>
-  <si>
-    <t>Pregnancy Status Effective Date</t>
-  </si>
-  <si>
-    <t>Pregnancy Status Value</t>
+    <t>MedicationRequest.reportedBoolean</t>
+  </si>
+  <si>
+    <t>Medication Reported</t>
+  </si>
+  <si>
+    <t>http://loinc.org^8289-1^</t>
+  </si>
+  <si>
+    <t>Pediatric Head Occipital Frontal Circumference Code</t>
+  </si>
+  <si>
+    <t>Pediatric Head Occipital Frontal Circumference Status</t>
+  </si>
+  <si>
+    <t>Pediatric Head Occipital Frontal Circumference Value</t>
+  </si>
+  <si>
+    <t>Pediatric BMI Status</t>
+  </si>
+  <si>
+    <t>Pediatric BMI Value</t>
+  </si>
+  <si>
+    <t>Pediatric BMI Category</t>
+  </si>
+  <si>
+    <t>http://terminology.hl7.org/CodeSystem/observation-category^vital-signs</t>
+  </si>
+  <si>
+    <t>Pediatric BMI EffectiveDateTIme</t>
+  </si>
+  <si>
+    <t>Pediatric BMI Code</t>
+  </si>
+  <si>
+    <t>http://loinc.org^59576-9</t>
+  </si>
+  <si>
+    <t>Pediatric Head Occipital Frontal Circumference Category</t>
+  </si>
+  <si>
+    <t>Observation.category</t>
+  </si>
+  <si>
+    <t>Pediatric Head Occipital Frontal Circumference Effective Date</t>
+  </si>
+  <si>
+    <t>PregnancyStatus time issued</t>
+  </si>
+  <si>
+    <t>PregnancyStatus Effective Date</t>
+  </si>
+  <si>
+    <t>PregnancyStatus Value</t>
+  </si>
+  <si>
+    <t>SmokingStatus time issued</t>
+  </si>
+  <si>
+    <t>SmokingStatus Effective Date</t>
+  </si>
+  <si>
+    <t>SmokingStatus Value</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/us/core/StructureDefinition/us-core-observation-pregnancystatus</t>
   </si>
 </sst>
 </file>
@@ -2027,7 +2084,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="28" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="29" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="133">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2317,6 +2374,7 @@
     <xf numFmtId="0" fontId="4" fillId="22" borderId="2" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="3" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2326,24 +2384,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="21" borderId="0" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" xfId="5" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="4" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -2353,7 +2411,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="3" applyBorder="1"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="5" xfId="3" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Explanatory Text" xfId="2" builtinId="53"/>
@@ -2773,36 +2833,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="20" x14ac:dyDescent="0.2">
-      <c r="A1" s="125" t="s">
+      <c r="A1" s="128" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="125"/>
+      <c r="B1" s="128"/>
     </row>
     <row r="2" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="123" t="s">
+      <c r="A2" s="125" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="123"/>
-      <c r="C2" s="123"/>
+      <c r="B2" s="125"/>
+      <c r="C2" s="125"/>
     </row>
     <row r="3" spans="1:3" ht="103.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="124" t="s">
+      <c r="A3" s="127" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="124"/>
+      <c r="B3" s="127"/>
     </row>
     <row r="4" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="122" t="s">
+      <c r="A4" s="126" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="122"/>
-      <c r="C4" s="122"/>
+      <c r="B4" s="126"/>
+      <c r="C4" s="126"/>
     </row>
     <row r="5" spans="1:3" ht="40.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="127" t="s">
+      <c r="A5" s="124" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="127"/>
+      <c r="B5" s="124"/>
     </row>
     <row r="6" spans="1:3" ht="64" x14ac:dyDescent="0.2">
       <c r="A6" s="97" t="s">
@@ -2837,35 +2897,35 @@
       </c>
     </row>
     <row r="10" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="123" t="s">
+      <c r="A10" s="125" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="123"/>
-      <c r="C10" s="123"/>
+      <c r="B10" s="125"/>
+      <c r="C10" s="125"/>
     </row>
     <row r="11" spans="1:3" ht="37.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="124" t="s">
+      <c r="A11" s="127" t="s">
         <v>300</v>
       </c>
-      <c r="B11" s="124"/>
+      <c r="B11" s="127"/>
     </row>
     <row r="12" spans="1:3" ht="37.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="126" t="s">
+      <c r="A12" s="123" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="126"/>
+      <c r="B12" s="123"/>
     </row>
     <row r="13" spans="1:3" ht="37.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="126" t="s">
+      <c r="A13" s="123" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="126"/>
+      <c r="B13" s="123"/>
     </row>
     <row r="14" spans="1:3" ht="37.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="126" t="s">
+      <c r="A14" s="123" t="s">
         <v>303</v>
       </c>
-      <c r="B14" s="126"/>
+      <c r="B14" s="123"/>
     </row>
     <row r="15" spans="1:3" ht="36" x14ac:dyDescent="0.2">
       <c r="A15" s="98" t="s">
@@ -2922,16 +2982,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A11:B11"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A11:B11"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A6" location="ResourceDefinitions!A1" display="ResourceDefinitions" xr:uid="{21E4973D-DCF1-4F08-A5DE-B12BC88A3D35}"/>
@@ -3881,7 +3941,7 @@
       <c r="DW6" s="14"/>
     </row>
     <row r="7" spans="1:127" x14ac:dyDescent="0.2">
-      <c r="A7" s="120"/>
+      <c r="A7" s="121"/>
       <c r="B7" s="5"/>
       <c r="C7" s="16"/>
       <c r="D7" s="17"/>
@@ -3991,7 +4051,7 @@
       <c r="DD7" s="19"/>
     </row>
     <row r="8" spans="1:127" x14ac:dyDescent="0.2">
-      <c r="A8" s="120"/>
+      <c r="A8" s="121"/>
       <c r="B8" s="5"/>
       <c r="C8" s="20"/>
       <c r="CK8" s="15"/>
@@ -4005,7 +4065,7 @@
       <c r="DD8" s="21"/>
     </row>
     <row r="9" spans="1:127" x14ac:dyDescent="0.2">
-      <c r="A9" s="120"/>
+      <c r="A9" s="121"/>
       <c r="B9" s="5"/>
       <c r="C9" s="20"/>
       <c r="CK9" s="15"/>
@@ -4019,7 +4079,7 @@
       <c r="DD9" s="21"/>
     </row>
     <row r="10" spans="1:127" x14ac:dyDescent="0.2">
-      <c r="A10" s="120"/>
+      <c r="A10" s="121"/>
       <c r="B10" s="5"/>
       <c r="C10" s="20"/>
       <c r="CK10" s="15"/>
@@ -4033,7 +4093,7 @@
       <c r="DD10" s="21"/>
     </row>
     <row r="11" spans="1:127" x14ac:dyDescent="0.2">
-      <c r="A11" s="120"/>
+      <c r="A11" s="121"/>
       <c r="B11" s="5"/>
       <c r="C11" s="20"/>
       <c r="CK11" s="15"/>
@@ -4047,7 +4107,7 @@
       <c r="DD11" s="21"/>
     </row>
     <row r="12" spans="1:127" x14ac:dyDescent="0.2">
-      <c r="A12" s="120"/>
+      <c r="A12" s="121"/>
       <c r="B12" s="5"/>
       <c r="C12" s="20"/>
       <c r="CK12" s="15"/>
@@ -4061,7 +4121,7 @@
       <c r="DD12" s="21"/>
     </row>
     <row r="13" spans="1:127" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="120"/>
+      <c r="A13" s="121"/>
       <c r="B13" s="5"/>
       <c r="C13" s="20"/>
       <c r="CK13" s="15"/>
@@ -4075,7 +4135,7 @@
       <c r="DD13" s="21"/>
     </row>
     <row r="14" spans="1:127" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="120"/>
+      <c r="A14" s="121"/>
       <c r="B14" s="5"/>
       <c r="C14" s="20"/>
       <c r="CK14" s="15"/>
@@ -4089,7 +4149,7 @@
       <c r="DD14" s="21"/>
     </row>
     <row r="15" spans="1:127" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="120"/>
+      <c r="A15" s="121"/>
       <c r="B15" s="5"/>
       <c r="C15" s="20"/>
       <c r="CK15" s="15"/>
@@ -4103,7 +4163,7 @@
       <c r="DD15" s="21"/>
     </row>
     <row r="16" spans="1:127" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="121"/>
+      <c r="A16" s="122"/>
       <c r="B16" s="6"/>
       <c r="C16" s="9"/>
       <c r="D16" s="10"/>
@@ -4223,7 +4283,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D010D53-A2B8-4D7D-8239-2883E618B035}">
-  <dimension ref="A1:EO16"/>
+  <dimension ref="A1:EV16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="30" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.6640625" customWidth="1"/>
@@ -4232,12 +4292,13 @@
     <col min="28" max="29" width="30" customWidth="1"/>
     <col min="31" max="99" width="30" customWidth="1"/>
     <col min="100" max="100" width="43" customWidth="1"/>
-    <col min="101" max="101" width="30" customWidth="1"/>
-    <col min="102" max="102" width="43.6640625" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="30" customWidth="1"/>
+    <col min="101" max="102" width="30" customWidth="1"/>
+    <col min="103" max="104" width="43.6640625" bestFit="1" customWidth="1"/>
+    <col min="105" max="106" width="43.6640625" customWidth="1"/>
+    <col min="107" max="107" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:145" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:152" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="25" t="s">
         <v>31</v>
       </c>
@@ -4343,21 +4404,21 @@
       <c r="CU1" s="83"/>
       <c r="CV1" s="83"/>
       <c r="CW1" s="83"/>
-      <c r="CX1" s="84"/>
+      <c r="CX1" s="83"/>
       <c r="CY1" s="84"/>
       <c r="CZ1" s="84"/>
       <c r="DA1" s="84"/>
-      <c r="DB1" s="85"/>
-      <c r="DC1" s="85"/>
-      <c r="DD1" s="86"/>
-      <c r="DE1" s="86"/>
+      <c r="DB1" s="84"/>
+      <c r="DC1" s="84"/>
+      <c r="DD1" s="85"/>
+      <c r="DE1" s="85"/>
       <c r="DF1" s="86"/>
-      <c r="DG1" s="85"/>
-      <c r="DH1" s="85"/>
+      <c r="DG1" s="86"/>
+      <c r="DH1" s="86"/>
       <c r="DI1" s="85"/>
       <c r="DJ1" s="85"/>
-      <c r="DK1" s="91"/>
-      <c r="DL1" s="91"/>
+      <c r="DK1" s="85"/>
+      <c r="DL1" s="85"/>
       <c r="DM1" s="91"/>
       <c r="DN1" s="91"/>
       <c r="DO1" s="91"/>
@@ -4371,28 +4432,35 @@
       <c r="DW1" s="91"/>
       <c r="DX1" s="91"/>
       <c r="DY1" s="91"/>
-      <c r="DZ1" s="81" t="s">
-        <v>405</v>
-      </c>
-      <c r="EA1" s="81"/>
-      <c r="EB1" s="81"/>
+      <c r="DZ1" s="91"/>
+      <c r="EA1" s="91"/>
+      <c r="EB1" s="81" t="s">
+        <v>404</v>
+      </c>
       <c r="EC1" s="81"/>
-      <c r="ED1" s="82" t="s">
-        <v>405</v>
-      </c>
-      <c r="EE1" s="82"/>
-      <c r="EF1" s="82"/>
+      <c r="ED1" s="81"/>
+      <c r="EE1" s="81"/>
+      <c r="EF1" s="82" t="s">
+        <v>404</v>
+      </c>
       <c r="EG1" s="82"/>
       <c r="EH1" s="82"/>
       <c r="EI1" s="82"/>
-      <c r="EJ1" s="65"/>
-      <c r="EK1" s="65"/>
+      <c r="EJ1" s="82"/>
+      <c r="EK1" s="82"/>
       <c r="EL1" s="65"/>
       <c r="EM1" s="65"/>
       <c r="EN1" s="65"/>
       <c r="EO1" s="65"/>
+      <c r="EP1" s="65"/>
+      <c r="EQ1" s="65"/>
+      <c r="ER1" s="84"/>
+      <c r="ES1" s="84"/>
+      <c r="ET1" s="84"/>
+      <c r="EU1" s="84"/>
+      <c r="EV1" s="84"/>
     </row>
-    <row r="2" spans="1:145" s="2" customFormat="1" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:152" s="2" customFormat="1" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="29" t="s">
         <v>33</v>
       </c>
@@ -4457,10 +4525,10 @@
         <v>61</v>
       </c>
       <c r="V2" s="38" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="W2" s="38" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="X2" s="38" t="s">
         <v>62</v>
@@ -4652,7 +4720,7 @@
         <v>115</v>
       </c>
       <c r="CI2" s="62" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="CJ2" s="62" t="s">
         <v>117</v>
@@ -4685,10 +4753,10 @@
         <v>119</v>
       </c>
       <c r="CT2" s="64" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="CU2" s="64" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="CV2" s="64" t="s">
         <v>121</v>
@@ -4696,140 +4764,161 @@
       <c r="CW2" s="64" t="s">
         <v>122</v>
       </c>
-      <c r="CX2" s="66" t="s">
+      <c r="CX2" s="64" t="s">
+        <v>422</v>
+      </c>
+      <c r="CY2" s="66" t="s">
+        <v>436</v>
+      </c>
+      <c r="CZ2" s="66" t="s">
         <v>95</v>
       </c>
-      <c r="CY2" s="66" t="s">
+      <c r="DA2" s="66" t="s">
+        <v>102</v>
+      </c>
+      <c r="DB2" s="66" t="s">
+        <v>103</v>
+      </c>
+      <c r="DC2" s="66" t="s">
         <v>104</v>
       </c>
-      <c r="CZ2" s="66" t="s">
+      <c r="DD2" s="68" t="s">
+        <v>124</v>
+      </c>
+      <c r="DE2" s="68" t="s">
+        <v>125</v>
+      </c>
+      <c r="DF2" s="68" t="s">
+        <v>126</v>
+      </c>
+      <c r="DG2" s="68" t="s">
+        <v>127</v>
+      </c>
+      <c r="DH2" s="68" t="s">
+        <v>128</v>
+      </c>
+      <c r="DI2" s="68" t="s">
+        <v>129</v>
+      </c>
+      <c r="DJ2" s="68" t="s">
+        <v>130</v>
+      </c>
+      <c r="DK2" s="68" t="s">
+        <v>131</v>
+      </c>
+      <c r="DL2" s="68" t="s">
+        <v>132</v>
+      </c>
+      <c r="DM2" s="91" t="s">
+        <v>102</v>
+      </c>
+      <c r="DN2" s="91" t="s">
+        <v>95</v>
+      </c>
+      <c r="DO2" s="91" t="s">
+        <v>315</v>
+      </c>
+      <c r="DP2" s="91" t="s">
+        <v>103</v>
+      </c>
+      <c r="DQ2" s="91" t="s">
         <v>104</v>
       </c>
-      <c r="DA2" s="66" t="s">
-        <v>123</v>
-      </c>
-      <c r="DB2" s="68" t="s">
-        <v>124</v>
-      </c>
-      <c r="DC2" s="68" t="s">
-        <v>125</v>
-      </c>
-      <c r="DD2" s="68" t="s">
-        <v>126</v>
-      </c>
-      <c r="DE2" s="68" t="s">
-        <v>127</v>
-      </c>
-      <c r="DF2" s="68" t="s">
-        <v>128</v>
-      </c>
-      <c r="DG2" s="68" t="s">
-        <v>129</v>
-      </c>
-      <c r="DH2" s="68" t="s">
-        <v>130</v>
-      </c>
-      <c r="DI2" s="68" t="s">
-        <v>131</v>
-      </c>
-      <c r="DJ2" s="68" t="s">
-        <v>132</v>
-      </c>
-      <c r="DK2" s="91" t="s">
+      <c r="DR2" s="91" t="s">
+        <v>97</v>
+      </c>
+      <c r="DS2" s="91" t="s">
+        <v>105</v>
+      </c>
+      <c r="DT2" s="91" t="s">
+        <v>106</v>
+      </c>
+      <c r="DU2" s="91" t="s">
+        <v>107</v>
+      </c>
+      <c r="DV2" s="91" t="s">
+        <v>108</v>
+      </c>
+      <c r="DW2" s="91" t="s">
+        <v>109</v>
+      </c>
+      <c r="DX2" s="91" t="s">
+        <v>110</v>
+      </c>
+      <c r="DY2" s="91" t="s">
+        <v>111</v>
+      </c>
+      <c r="DZ2" s="91" t="s">
+        <v>112</v>
+      </c>
+      <c r="EA2" s="91" t="s">
+        <v>113</v>
+      </c>
+      <c r="EB2" s="60" t="s">
+        <v>388</v>
+      </c>
+      <c r="EC2" s="60" t="s">
+        <v>390</v>
+      </c>
+      <c r="ED2" s="60" t="s">
+        <v>392</v>
+      </c>
+      <c r="EE2" s="60" t="s">
+        <v>395</v>
+      </c>
+      <c r="EF2" s="62" t="s">
+        <v>315</v>
+      </c>
+      <c r="EG2" s="62" t="s">
         <v>102</v>
       </c>
-      <c r="DL2" s="91" t="s">
+      <c r="EH2" s="62" t="s">
+        <v>411</v>
+      </c>
+      <c r="EI2" s="62" t="s">
+        <v>97</v>
+      </c>
+      <c r="EJ2" s="62" t="s">
+        <v>414</v>
+      </c>
+      <c r="EK2" s="62" t="s">
+        <v>415</v>
+      </c>
+      <c r="EL2" s="64" t="s">
         <v>95</v>
       </c>
-      <c r="DM2" s="91" t="s">
+      <c r="EM2" s="64" t="s">
+        <v>102</v>
+      </c>
+      <c r="EN2" s="64" t="s">
         <v>315</v>
       </c>
-      <c r="DN2" s="91" t="s">
+      <c r="EO2" s="64" t="s">
+        <v>96</v>
+      </c>
+      <c r="EP2" s="64" t="s">
         <v>103</v>
       </c>
-      <c r="DO2" s="91" t="s">
+      <c r="EQ2" s="64" t="s">
+        <v>97</v>
+      </c>
+      <c r="ER2" s="66" t="s">
+        <v>436</v>
+      </c>
+      <c r="ES2" s="66" t="s">
+        <v>95</v>
+      </c>
+      <c r="ET2" s="66" t="s">
+        <v>102</v>
+      </c>
+      <c r="EU2" s="66" t="s">
+        <v>103</v>
+      </c>
+      <c r="EV2" s="66" t="s">
         <v>104</v>
       </c>
-      <c r="DP2" s="91" t="s">
-        <v>97</v>
-      </c>
-      <c r="DQ2" s="91" t="s">
-        <v>105</v>
-      </c>
-      <c r="DR2" s="91" t="s">
-        <v>106</v>
-      </c>
-      <c r="DS2" s="91" t="s">
-        <v>107</v>
-      </c>
-      <c r="DT2" s="91" t="s">
-        <v>108</v>
-      </c>
-      <c r="DU2" s="91" t="s">
-        <v>109</v>
-      </c>
-      <c r="DV2" s="91" t="s">
-        <v>110</v>
-      </c>
-      <c r="DW2" s="91" t="s">
-        <v>111</v>
-      </c>
-      <c r="DX2" s="91" t="s">
-        <v>112</v>
-      </c>
-      <c r="DY2" s="91" t="s">
-        <v>113</v>
-      </c>
-      <c r="DZ2" s="60" t="s">
-        <v>389</v>
-      </c>
-      <c r="EA2" s="60" t="s">
-        <v>391</v>
-      </c>
-      <c r="EB2" s="60" t="s">
-        <v>393</v>
-      </c>
-      <c r="EC2" s="60" t="s">
-        <v>396</v>
-      </c>
-      <c r="ED2" s="62" t="s">
-        <v>315</v>
-      </c>
-      <c r="EE2" s="62" t="s">
-        <v>102</v>
-      </c>
-      <c r="EF2" s="62" t="s">
-        <v>412</v>
-      </c>
-      <c r="EG2" s="62" t="s">
-        <v>97</v>
-      </c>
-      <c r="EH2" s="62" t="s">
-        <v>415</v>
-      </c>
-      <c r="EI2" s="62" t="s">
-        <v>416</v>
-      </c>
-      <c r="EJ2" s="64" t="s">
-        <v>95</v>
-      </c>
-      <c r="EK2" s="64" t="s">
-        <v>102</v>
-      </c>
-      <c r="EL2" s="64" t="s">
-        <v>315</v>
-      </c>
-      <c r="EM2" s="64" t="s">
-        <v>96</v>
-      </c>
-      <c r="EN2" s="64" t="s">
-        <v>103</v>
-      </c>
-      <c r="EO2" s="64" t="s">
-        <v>97</v>
-      </c>
     </row>
-    <row r="3" spans="1:145" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:152" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="31" t="s">
         <v>35</v>
       </c>
@@ -5129,140 +5218,161 @@
       <c r="CW3" s="64" t="s">
         <v>135</v>
       </c>
-      <c r="CX3" s="66" t="s">
+      <c r="CX3" s="64" t="s">
+        <v>138</v>
+      </c>
+      <c r="CY3" s="66" t="s">
         <v>134</v>
       </c>
-      <c r="CY3" s="66" t="s">
+      <c r="CZ3" s="66" t="s">
+        <v>134</v>
+      </c>
+      <c r="DA3" s="66" t="s">
+        <v>16</v>
+      </c>
+      <c r="DB3" s="66" t="s">
+        <v>139</v>
+      </c>
+      <c r="DC3" s="66" t="s">
         <v>142</v>
-      </c>
-      <c r="CZ3" s="66" t="s">
-        <v>142</v>
-      </c>
-      <c r="DA3" s="66" t="s">
-        <v>140</v>
-      </c>
-      <c r="DB3" s="68" t="s">
-        <v>135</v>
-      </c>
-      <c r="DC3" s="68" t="s">
-        <v>149</v>
       </c>
       <c r="DD3" s="68" t="s">
         <v>135</v>
       </c>
       <c r="DE3" s="68" t="s">
+        <v>149</v>
+      </c>
+      <c r="DF3" s="68" t="s">
         <v>135</v>
       </c>
-      <c r="DF3" s="68" t="s">
+      <c r="DG3" s="68" t="s">
+        <v>135</v>
+      </c>
+      <c r="DH3" s="68" t="s">
         <v>139</v>
       </c>
-      <c r="DG3" s="68" t="s">
+      <c r="DI3" s="68" t="s">
         <v>139</v>
       </c>
-      <c r="DH3" s="68" t="s">
+      <c r="DJ3" s="68" t="s">
         <v>135</v>
       </c>
-      <c r="DI3" s="68" t="s">
+      <c r="DK3" s="68" t="s">
         <v>135</v>
       </c>
-      <c r="DJ3" s="68" t="s">
+      <c r="DL3" s="68" t="s">
         <v>16</v>
-      </c>
-      <c r="DK3" s="91" t="s">
-        <v>16</v>
-      </c>
-      <c r="DL3" s="91" t="s">
-        <v>134</v>
       </c>
       <c r="DM3" s="91" t="s">
         <v>16</v>
       </c>
       <c r="DN3" s="91" t="s">
+        <v>134</v>
+      </c>
+      <c r="DO3" s="91" t="s">
+        <v>16</v>
+      </c>
+      <c r="DP3" s="91" t="s">
         <v>139</v>
       </c>
-      <c r="DO3" s="91" t="s">
+      <c r="DQ3" s="91" t="s">
         <v>142</v>
       </c>
-      <c r="DP3" s="91" t="s">
+      <c r="DR3" s="91" t="s">
         <v>16</v>
       </c>
-      <c r="DQ3" s="91" t="s">
+      <c r="DS3" s="91" t="s">
         <v>135</v>
       </c>
-      <c r="DR3" s="91" t="s">
+      <c r="DT3" s="91" t="s">
         <v>138</v>
       </c>
-      <c r="DS3" s="91" t="s">
+      <c r="DU3" s="91" t="s">
         <v>143</v>
       </c>
-      <c r="DT3" s="91" t="s">
+      <c r="DV3" s="91" t="s">
         <v>144</v>
       </c>
-      <c r="DU3" s="91" t="s">
+      <c r="DW3" s="91" t="s">
         <v>145</v>
       </c>
-      <c r="DV3" s="91" t="s">
+      <c r="DX3" s="91" t="s">
         <v>146</v>
       </c>
-      <c r="DW3" s="91" t="s">
+      <c r="DY3" s="91" t="s">
         <v>139</v>
       </c>
-      <c r="DX3" s="91" t="s">
+      <c r="DZ3" s="91" t="s">
         <v>147</v>
       </c>
-      <c r="DY3" s="91" t="s">
+      <c r="EA3" s="91" t="s">
         <v>16</v>
       </c>
-      <c r="DZ3" s="60" t="s">
+      <c r="EB3" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="EA3" s="60" t="s">
+      <c r="EC3" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="EB3" s="60" t="s">
+      <c r="ED3" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="EC3" s="60" t="s">
+      <c r="EE3" s="60" t="s">
         <v>139</v>
       </c>
-      <c r="ED3" s="62" t="s">
-        <v>408</v>
-      </c>
-      <c r="EE3" s="62" t="s">
+      <c r="EF3" s="62" t="s">
+        <v>407</v>
+      </c>
+      <c r="EG3" s="62" t="s">
         <v>134</v>
       </c>
-      <c r="EF3" s="62" t="s">
+      <c r="EH3" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="EG3" s="62" t="s">
+      <c r="EI3" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="EH3" s="62" t="s">
+      <c r="EJ3" s="62" t="s">
         <v>139</v>
       </c>
-      <c r="EI3" s="62" t="s">
+      <c r="EK3" s="62" t="s">
         <v>139</v>
       </c>
-      <c r="EJ3" s="64" t="s">
+      <c r="EL3" s="64" t="s">
         <v>134</v>
       </c>
-      <c r="EK3" s="64" t="s">
+      <c r="EM3" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="EL3" s="64" t="s">
+      <c r="EN3" s="64" t="s">
         <v>18</v>
       </c>
-      <c r="EM3" s="64" t="s">
+      <c r="EO3" s="64" t="s">
         <v>141</v>
       </c>
-      <c r="EN3" s="64" t="s">
+      <c r="EP3" s="64" t="s">
         <v>139</v>
       </c>
-      <c r="EO3" s="64" t="s">
+      <c r="EQ3" s="64" t="s">
         <v>16</v>
       </c>
+      <c r="ER3" s="66" t="s">
+        <v>134</v>
+      </c>
+      <c r="ES3" s="66" t="s">
+        <v>134</v>
+      </c>
+      <c r="ET3" s="66" t="s">
+        <v>142</v>
+      </c>
+      <c r="EU3" s="66" t="s">
+        <v>148</v>
+      </c>
+      <c r="EV3" s="66" t="s">
+        <v>142</v>
+      </c>
     </row>
-    <row r="4" spans="1:145" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:152" ht="52.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="32" t="s">
         <v>37</v>
       </c>
@@ -5448,26 +5558,28 @@
       </c>
       <c r="CV4" s="64"/>
       <c r="CW4" s="64"/>
-      <c r="CX4" s="67"/>
-      <c r="CY4" s="67"/>
+      <c r="CX4" s="64"/>
+      <c r="CY4" s="67" t="s">
+        <v>320</v>
+      </c>
       <c r="CZ4" s="67"/>
       <c r="DA4" s="67"/>
-      <c r="DB4" s="69"/>
-      <c r="DC4" s="69"/>
+      <c r="DB4" s="67"/>
+      <c r="DC4" s="67"/>
       <c r="DD4" s="69"/>
       <c r="DE4" s="69"/>
       <c r="DF4" s="69"/>
       <c r="DG4" s="69"/>
       <c r="DH4" s="69"/>
       <c r="DI4" s="69"/>
-      <c r="DJ4" s="69" t="s">
+      <c r="DJ4" s="69"/>
+      <c r="DK4" s="69"/>
+      <c r="DL4" s="69" t="s">
         <v>183</v>
       </c>
-      <c r="DK4" s="91" t="s">
+      <c r="DM4" s="91" t="s">
         <v>184</v>
       </c>
-      <c r="DL4" s="91"/>
-      <c r="DM4" s="91"/>
       <c r="DN4" s="91"/>
       <c r="DO4" s="91"/>
       <c r="DP4" s="91"/>
@@ -5480,32 +5592,41 @@
       <c r="DW4" s="91"/>
       <c r="DX4" s="91"/>
       <c r="DY4" s="91"/>
-      <c r="DZ4" s="61"/>
-      <c r="EA4" s="61"/>
+      <c r="DZ4" s="91"/>
+      <c r="EA4" s="91"/>
       <c r="EB4" s="61"/>
-      <c r="EC4" s="60"/>
-      <c r="ED4" s="63"/>
-      <c r="EE4" s="63"/>
+      <c r="EC4" s="61"/>
+      <c r="ED4" s="61"/>
+      <c r="EE4" s="60"/>
       <c r="EF4" s="63"/>
-      <c r="EG4" s="62"/>
-      <c r="EH4" s="62"/>
+      <c r="EG4" s="63"/>
+      <c r="EH4" s="63"/>
       <c r="EI4" s="62"/>
-      <c r="EJ4" s="65" t="s">
+      <c r="EJ4" s="62"/>
+      <c r="EK4" s="62"/>
+      <c r="EL4" s="65" t="s">
         <v>172</v>
       </c>
-      <c r="EK4" s="65" t="s">
+      <c r="EM4" s="65" t="s">
         <v>177</v>
       </c>
-      <c r="EL4" s="65" t="s">
+      <c r="EN4" s="65" t="s">
         <v>320</v>
       </c>
-      <c r="EM4" s="65"/>
-      <c r="EN4" s="65"/>
-      <c r="EO4" s="65" t="s">
+      <c r="EO4" s="65"/>
+      <c r="EP4" s="65"/>
+      <c r="EQ4" s="65" t="s">
         <v>173</v>
       </c>
+      <c r="ER4" s="67" t="s">
+        <v>320</v>
+      </c>
+      <c r="ES4" s="67"/>
+      <c r="ET4" s="67"/>
+      <c r="EU4" s="67"/>
+      <c r="EV4" s="67"/>
     </row>
-    <row r="5" spans="1:145" ht="65.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:152" ht="65.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="27" t="s">
         <v>39</v>
       </c>
@@ -5803,23 +5924,23 @@
       <c r="CW5" s="64" t="s">
         <v>199</v>
       </c>
-      <c r="CX5" s="67" t="s">
-        <v>200</v>
+      <c r="CX5" s="64" t="s">
+        <v>199</v>
       </c>
       <c r="CY5" s="67" t="s">
         <v>200</v>
       </c>
-      <c r="CZ5" s="66" t="s">
+      <c r="CZ5" s="67" t="s">
         <v>200</v>
       </c>
-      <c r="DA5" s="66" t="s">
-        <v>201</v>
-      </c>
-      <c r="DB5" s="68" t="s">
-        <v>202</v>
-      </c>
-      <c r="DC5" s="68" t="s">
-        <v>202</v>
+      <c r="DA5" s="67" t="s">
+        <v>200</v>
+      </c>
+      <c r="DB5" s="67" t="s">
+        <v>200</v>
+      </c>
+      <c r="DC5" s="67" t="s">
+        <v>200</v>
       </c>
       <c r="DD5" s="68" t="s">
         <v>202</v>
@@ -5842,11 +5963,11 @@
       <c r="DJ5" s="68" t="s">
         <v>202</v>
       </c>
-      <c r="DK5" s="91" t="s">
-        <v>203</v>
-      </c>
-      <c r="DL5" s="91" t="s">
-        <v>203</v>
+      <c r="DK5" s="68" t="s">
+        <v>202</v>
+      </c>
+      <c r="DL5" s="68" t="s">
+        <v>202</v>
       </c>
       <c r="DM5" s="91" t="s">
         <v>203</v>
@@ -5869,10 +5990,10 @@
       <c r="DS5" s="91" t="s">
         <v>203</v>
       </c>
-      <c r="DT5" s="118" t="s">
+      <c r="DT5" s="91" t="s">
         <v>203</v>
       </c>
-      <c r="DU5" s="118" t="s">
+      <c r="DU5" s="91" t="s">
         <v>203</v>
       </c>
       <c r="DV5" s="118" t="s">
@@ -5887,56 +6008,77 @@
       <c r="DY5" s="118" t="s">
         <v>203</v>
       </c>
-      <c r="DZ5" s="61" t="s">
-        <v>388</v>
-      </c>
-      <c r="EA5" s="61" t="s">
-        <v>388</v>
+      <c r="DZ5" s="118" t="s">
+        <v>203</v>
+      </c>
+      <c r="EA5" s="118" t="s">
+        <v>203</v>
       </c>
       <c r="EB5" s="61" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="EC5" s="61" t="s">
-        <v>388</v>
-      </c>
-      <c r="ED5" s="63" t="s">
-        <v>407</v>
-      </c>
-      <c r="EE5" s="63" t="s">
-        <v>407</v>
+        <v>387</v>
+      </c>
+      <c r="ED5" s="61" t="s">
+        <v>387</v>
+      </c>
+      <c r="EE5" s="61" t="s">
+        <v>387</v>
       </c>
       <c r="EF5" s="63" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="EG5" s="63" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="EH5" s="63" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="EI5" s="63" t="s">
-        <v>407</v>
-      </c>
-      <c r="EJ5" s="64" t="s">
-        <v>195</v>
-      </c>
-      <c r="EK5" s="64" t="s">
-        <v>195</v>
+        <v>406</v>
+      </c>
+      <c r="EJ5" s="63" t="s">
+        <v>406</v>
+      </c>
+      <c r="EK5" s="63" t="s">
+        <v>406</v>
       </c>
       <c r="EL5" s="65" t="s">
-        <v>195</v>
-      </c>
-      <c r="EM5" s="64" t="s">
-        <v>195</v>
-      </c>
-      <c r="EN5" s="64" t="s">
-        <v>195</v>
-      </c>
-      <c r="EO5" s="64" t="s">
-        <v>195</v>
+        <v>444</v>
+      </c>
+      <c r="EM5" s="65" t="s">
+        <v>444</v>
+      </c>
+      <c r="EN5" s="65" t="s">
+        <v>444</v>
+      </c>
+      <c r="EO5" s="65" t="s">
+        <v>444</v>
+      </c>
+      <c r="EP5" s="65" t="s">
+        <v>444</v>
+      </c>
+      <c r="EQ5" s="65" t="s">
+        <v>444</v>
+      </c>
+      <c r="ER5" s="67" t="s">
+        <v>200</v>
+      </c>
+      <c r="ES5" s="67" t="s">
+        <v>198</v>
+      </c>
+      <c r="ET5" s="67" t="s">
+        <v>198</v>
+      </c>
+      <c r="EU5" s="67" t="s">
+        <v>198</v>
+      </c>
+      <c r="EV5" s="67" t="s">
+        <v>198</v>
       </c>
     </row>
-    <row r="6" spans="1:145" s="2" customFormat="1" ht="52.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:152" s="2" customFormat="1" ht="52.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="34" t="s">
         <v>41</v>
       </c>
@@ -6010,7 +6152,7 @@
         <v>224</v>
       </c>
       <c r="Y6" s="89" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="Z6" s="89" t="s">
         <v>225</v>
@@ -6154,13 +6296,13 @@
         <v>329</v>
       </c>
       <c r="BU6" s="89" t="s">
-        <v>265</v>
+        <v>441</v>
       </c>
       <c r="BV6" s="89" t="s">
-        <v>386</v>
+        <v>442</v>
       </c>
       <c r="BW6" s="89" t="s">
-        <v>266</v>
+        <v>443</v>
       </c>
       <c r="BX6" s="89" t="s">
         <v>267</v>
@@ -6229,7 +6371,7 @@
         <v>280</v>
       </c>
       <c r="CT6" s="89" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="CU6" s="89" t="s">
         <v>281</v>
@@ -6241,59 +6383,59 @@
         <v>283</v>
       </c>
       <c r="CX6" s="89" t="s">
-        <v>330</v>
+        <v>423</v>
       </c>
       <c r="CY6" s="89" t="s">
-        <v>284</v>
+        <v>430</v>
       </c>
       <c r="CZ6" s="89" t="s">
-        <v>285</v>
+        <v>428</v>
       </c>
       <c r="DA6" s="89" t="s">
-        <v>286</v>
+        <v>433</v>
       </c>
       <c r="DB6" s="89" t="s">
+        <v>432</v>
+      </c>
+      <c r="DC6" s="89" t="s">
+        <v>429</v>
+      </c>
+      <c r="DD6" s="89" t="s">
         <v>287</v>
       </c>
-      <c r="DC6" s="89" t="s">
+      <c r="DE6" s="89" t="s">
         <v>288</v>
       </c>
-      <c r="DD6" s="89" t="s">
+      <c r="DF6" s="89" t="s">
         <v>289</v>
       </c>
-      <c r="DE6" s="89" t="s">
+      <c r="DG6" s="89" t="s">
         <v>290</v>
       </c>
-      <c r="DF6" s="89" t="s">
+      <c r="DH6" s="89" t="s">
         <v>291</v>
       </c>
-      <c r="DG6" s="89" t="s">
+      <c r="DI6" s="89" t="s">
         <v>292</v>
       </c>
-      <c r="DH6" s="89" t="s">
+      <c r="DJ6" s="89" t="s">
         <v>293</v>
       </c>
-      <c r="DI6" s="89" t="s">
+      <c r="DK6" s="89" t="s">
         <v>294</v>
       </c>
-      <c r="DJ6" s="90"/>
-      <c r="DK6" s="90" t="s">
+      <c r="DL6" s="90"/>
+      <c r="DM6" s="90" t="s">
         <v>295</v>
       </c>
-      <c r="DL6" s="90" t="s">
+      <c r="DN6" s="90" t="s">
+        <v>400</v>
+      </c>
+      <c r="DO6" s="90" t="s">
         <v>401</v>
       </c>
-      <c r="DM6" s="90" t="s">
-        <v>402</v>
-      </c>
-      <c r="DN6" s="90" t="s">
+      <c r="DP6" s="90" t="s">
         <v>296</v>
-      </c>
-      <c r="DO6" s="90" t="s">
-        <v>297</v>
-      </c>
-      <c r="DP6" s="90" t="s">
-        <v>297</v>
       </c>
       <c r="DQ6" s="90" t="s">
         <v>297</v>
@@ -6320,59 +6462,80 @@
         <v>297</v>
       </c>
       <c r="DY6" s="90" t="s">
+        <v>297</v>
+      </c>
+      <c r="DZ6" s="90" t="s">
+        <v>297</v>
+      </c>
+      <c r="EA6" s="90" t="s">
         <v>298</v>
       </c>
-      <c r="DZ6" s="89" t="s">
-        <v>390</v>
-      </c>
-      <c r="EA6" s="89" t="s">
-        <v>392</v>
-      </c>
       <c r="EB6" s="89" t="s">
+        <v>389</v>
+      </c>
+      <c r="EC6" s="89" t="s">
+        <v>391</v>
+      </c>
+      <c r="ED6" s="89" t="s">
+        <v>393</v>
+      </c>
+      <c r="EE6" s="89" t="s">
         <v>394</v>
       </c>
-      <c r="EC6" s="89" t="s">
-        <v>395</v>
-      </c>
-      <c r="ED6" s="89" t="s">
-        <v>406</v>
-      </c>
-      <c r="EE6" s="89" t="s">
-        <v>409</v>
-      </c>
       <c r="EF6" s="89" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
       <c r="EG6" s="89" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="EH6" s="89" t="s">
+        <v>410</v>
+      </c>
+      <c r="EI6" s="89" t="s">
+        <v>412</v>
+      </c>
+      <c r="EJ6" s="89" t="s">
+        <v>416</v>
+      </c>
+      <c r="EK6" s="89" t="s">
         <v>417</v>
       </c>
-      <c r="EI6" s="89" t="s">
+      <c r="EL6" s="89" t="s">
         <v>418</v>
       </c>
-      <c r="EJ6" s="89" t="s">
+      <c r="EM6" s="89" t="s">
         <v>419</v>
       </c>
-      <c r="EK6" s="89" t="s">
-        <v>420</v>
-      </c>
-      <c r="EL6" s="89" t="s">
-        <v>422</v>
-      </c>
-      <c r="EM6" s="89" t="s">
-        <v>423</v>
-      </c>
       <c r="EN6" s="89" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="EO6" s="89" t="s">
+        <v>438</v>
+      </c>
+      <c r="EP6" s="89" t="s">
+        <v>439</v>
+      </c>
+      <c r="EQ6" s="89" t="s">
+        <v>440</v>
+      </c>
+      <c r="ER6" s="89" t="s">
+        <v>435</v>
+      </c>
+      <c r="ES6" s="89" t="s">
+        <v>426</v>
+      </c>
+      <c r="ET6" s="89" t="s">
         <v>425</v>
       </c>
+      <c r="EU6" s="89" t="s">
+        <v>437</v>
+      </c>
+      <c r="EV6" s="89" t="s">
+        <v>427</v>
+      </c>
     </row>
-    <row r="7" spans="1:145" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="119"/>
+    <row r="7" spans="1:152" ht="32" x14ac:dyDescent="0.2">
+      <c r="A7" s="120"/>
       <c r="B7" s="5"/>
       <c r="C7" s="16"/>
       <c r="D7" s="17"/>
@@ -6473,15 +6636,19 @@
       <c r="CU7" s="18"/>
       <c r="CV7" s="17"/>
       <c r="CW7" s="17"/>
-      <c r="CX7" s="96" t="s">
+      <c r="CX7" s="17"/>
+      <c r="CY7" s="132" t="s">
+        <v>431</v>
+      </c>
+      <c r="CZ7" s="96" t="s">
         <v>331</v>
       </c>
-      <c r="CY7" s="17"/>
-      <c r="CZ7" s="17"/>
-      <c r="DA7" s="17"/>
-      <c r="DB7" s="18"/>
+      <c r="DA7" s="96" t="s">
+        <v>434</v>
+      </c>
+      <c r="DB7" s="96"/>
       <c r="DC7" s="17"/>
-      <c r="DD7" s="17"/>
+      <c r="DD7" s="18"/>
       <c r="DE7" s="17"/>
       <c r="DF7" s="17"/>
       <c r="DG7" s="17"/>
@@ -6502,34 +6669,47 @@
       <c r="DV7" s="17"/>
       <c r="DW7" s="17"/>
       <c r="DX7" s="17"/>
-      <c r="DY7" s="19"/>
+      <c r="DY7" s="17"/>
       <c r="DZ7" s="17"/>
-      <c r="EA7" s="17"/>
+      <c r="EA7" s="19"/>
       <c r="EB7" s="17"/>
       <c r="EC7" s="17"/>
-      <c r="ED7" s="131" t="s">
-        <v>414</v>
-      </c>
-      <c r="EE7" s="17" t="s">
-        <v>410</v>
-      </c>
-      <c r="EF7" s="17"/>
-      <c r="EG7" s="17"/>
+      <c r="ED7" s="17"/>
+      <c r="EE7" s="17"/>
+      <c r="EF7" s="119" t="s">
+        <v>413</v>
+      </c>
+      <c r="EG7" s="17" t="s">
+        <v>409</v>
+      </c>
       <c r="EH7" s="17"/>
       <c r="EI7" s="17"/>
       <c r="EJ7" s="17"/>
-      <c r="EK7" t="s">
-        <v>421</v>
-      </c>
-      <c r="EL7" s="131" t="s">
-        <v>414</v>
-      </c>
-      <c r="EM7" s="17"/>
-      <c r="EN7" s="17"/>
+      <c r="EK7" s="17"/>
+      <c r="EL7" s="17"/>
+      <c r="EM7" t="s">
+        <v>420</v>
+      </c>
+      <c r="EN7" s="119" t="s">
+        <v>413</v>
+      </c>
       <c r="EO7" s="17"/>
+      <c r="EP7" s="17"/>
+      <c r="EQ7" s="17"/>
+      <c r="ER7" s="132" t="s">
+        <v>431</v>
+      </c>
+      <c r="ES7" s="96" t="s">
+        <v>331</v>
+      </c>
+      <c r="ET7" s="17" t="s">
+        <v>424</v>
+      </c>
+      <c r="EU7" s="17"/>
+      <c r="EV7" s="17"/>
     </row>
-    <row r="8" spans="1:145" x14ac:dyDescent="0.2">
-      <c r="A8" s="120"/>
+    <row r="8" spans="1:152" x14ac:dyDescent="0.2">
+      <c r="A8" s="121"/>
       <c r="B8" s="5"/>
       <c r="C8" s="20"/>
       <c r="CG8" s="15"/>
@@ -6545,13 +6725,17 @@
       <c r="CQ8" s="15"/>
       <c r="CR8" s="15"/>
       <c r="CU8" s="8"/>
-      <c r="CX8" s="8"/>
-      <c r="DA8" s="15"/>
+      <c r="CY8" s="8"/>
+      <c r="CZ8" s="8"/>
+      <c r="DA8" s="8"/>
       <c r="DB8" s="8"/>
-      <c r="DY8" s="21"/>
+      <c r="DD8" s="8"/>
+      <c r="EA8" s="21"/>
+      <c r="ER8" s="8"/>
+      <c r="ES8" s="8"/>
     </row>
-    <row r="9" spans="1:145" x14ac:dyDescent="0.2">
-      <c r="A9" s="120"/>
+    <row r="9" spans="1:152" x14ac:dyDescent="0.2">
+      <c r="A9" s="121"/>
       <c r="B9" s="5"/>
       <c r="C9" s="20"/>
       <c r="CG9" s="15"/>
@@ -6567,13 +6751,16 @@
       <c r="CQ9" s="15"/>
       <c r="CR9" s="15"/>
       <c r="CU9" s="8"/>
-      <c r="CX9" s="8"/>
-      <c r="DA9" s="15"/>
+      <c r="CY9" s="8"/>
+      <c r="CZ9" s="8"/>
+      <c r="DA9" s="8"/>
       <c r="DB9" s="8"/>
-      <c r="DY9" s="21"/>
+      <c r="DD9" s="8"/>
+      <c r="EA9" s="21"/>
+      <c r="ER9" s="8"/>
     </row>
-    <row r="10" spans="1:145" x14ac:dyDescent="0.2">
-      <c r="A10" s="120"/>
+    <row r="10" spans="1:152" x14ac:dyDescent="0.2">
+      <c r="A10" s="121"/>
       <c r="B10" s="5"/>
       <c r="C10" s="20"/>
       <c r="CG10" s="15"/>
@@ -6589,13 +6776,16 @@
       <c r="CQ10" s="15"/>
       <c r="CR10" s="15"/>
       <c r="CU10" s="8"/>
-      <c r="CX10" s="8"/>
-      <c r="DA10" s="15"/>
+      <c r="CY10" s="8"/>
+      <c r="CZ10" s="8"/>
+      <c r="DA10" s="8"/>
       <c r="DB10" s="8"/>
-      <c r="DY10" s="21"/>
+      <c r="DD10" s="8"/>
+      <c r="EA10" s="21"/>
+      <c r="ER10" s="8"/>
     </row>
-    <row r="11" spans="1:145" x14ac:dyDescent="0.2">
-      <c r="A11" s="120"/>
+    <row r="11" spans="1:152" x14ac:dyDescent="0.2">
+      <c r="A11" s="121"/>
       <c r="B11" s="5"/>
       <c r="C11" s="20"/>
       <c r="CG11" s="15"/>
@@ -6611,13 +6801,16 @@
       <c r="CQ11" s="15"/>
       <c r="CR11" s="15"/>
       <c r="CU11" s="8"/>
-      <c r="CX11" s="8"/>
-      <c r="DA11" s="15"/>
+      <c r="CY11" s="8"/>
+      <c r="CZ11" s="8"/>
+      <c r="DA11" s="8"/>
       <c r="DB11" s="8"/>
-      <c r="DY11" s="21"/>
+      <c r="DD11" s="8"/>
+      <c r="EA11" s="21"/>
+      <c r="ER11" s="8"/>
     </row>
-    <row r="12" spans="1:145" x14ac:dyDescent="0.2">
-      <c r="A12" s="120"/>
+    <row r="12" spans="1:152" x14ac:dyDescent="0.2">
+      <c r="A12" s="121"/>
       <c r="B12" s="5"/>
       <c r="C12" s="20"/>
       <c r="CG12" s="15"/>
@@ -6633,13 +6826,16 @@
       <c r="CQ12" s="15"/>
       <c r="CR12" s="15"/>
       <c r="CU12" s="8"/>
-      <c r="CX12" s="8"/>
-      <c r="DA12" s="15"/>
+      <c r="CY12" s="8"/>
+      <c r="CZ12" s="8"/>
+      <c r="DA12" s="8"/>
       <c r="DB12" s="8"/>
-      <c r="DY12" s="21"/>
+      <c r="DD12" s="8"/>
+      <c r="EA12" s="21"/>
+      <c r="ER12" s="8"/>
     </row>
-    <row r="13" spans="1:145" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="120"/>
+    <row r="13" spans="1:152" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="121"/>
       <c r="B13" s="5"/>
       <c r="C13" s="20"/>
       <c r="CG13" s="15"/>
@@ -6655,13 +6851,16 @@
       <c r="CQ13" s="15"/>
       <c r="CR13" s="15"/>
       <c r="CU13" s="8"/>
-      <c r="CX13" s="8"/>
-      <c r="DA13" s="15"/>
+      <c r="CY13" s="8"/>
+      <c r="CZ13" s="8"/>
+      <c r="DA13" s="8"/>
       <c r="DB13" s="8"/>
-      <c r="DY13" s="21"/>
+      <c r="DD13" s="8"/>
+      <c r="EA13" s="21"/>
+      <c r="ER13" s="8"/>
     </row>
-    <row r="14" spans="1:145" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="120"/>
+    <row r="14" spans="1:152" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="121"/>
       <c r="B14" s="5"/>
       <c r="C14" s="20"/>
       <c r="CG14" s="15"/>
@@ -6677,13 +6876,16 @@
       <c r="CQ14" s="15"/>
       <c r="CR14" s="15"/>
       <c r="CU14" s="8"/>
-      <c r="CX14" s="8"/>
-      <c r="DA14" s="15"/>
+      <c r="CY14" s="8"/>
+      <c r="CZ14" s="8"/>
+      <c r="DA14" s="8"/>
       <c r="DB14" s="8"/>
-      <c r="DY14" s="21"/>
+      <c r="DD14" s="8"/>
+      <c r="EA14" s="21"/>
+      <c r="ER14" s="8"/>
     </row>
-    <row r="15" spans="1:145" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="120"/>
+    <row r="15" spans="1:152" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="121"/>
       <c r="B15" s="5"/>
       <c r="C15" s="20"/>
       <c r="CG15" s="15"/>
@@ -6699,13 +6901,16 @@
       <c r="CQ15" s="15"/>
       <c r="CR15" s="15"/>
       <c r="CU15" s="8"/>
-      <c r="CX15" s="8"/>
-      <c r="DA15" s="15"/>
+      <c r="CY15" s="8"/>
+      <c r="CZ15" s="8"/>
+      <c r="DA15" s="8"/>
       <c r="DB15" s="8"/>
-      <c r="DY15" s="21"/>
+      <c r="DD15" s="8"/>
+      <c r="EA15" s="21"/>
+      <c r="ER15" s="8"/>
     </row>
-    <row r="16" spans="1:145" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="121"/>
+    <row r="16" spans="1:152" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="122"/>
       <c r="B16" s="6"/>
       <c r="C16" s="9"/>
       <c r="D16" s="10"/>
@@ -6806,13 +7011,13 @@
       <c r="CU16" s="23"/>
       <c r="CV16" s="10"/>
       <c r="CW16" s="10"/>
-      <c r="CX16" s="23"/>
-      <c r="CY16" s="10"/>
-      <c r="CZ16" s="10"/>
-      <c r="DA16" s="22"/>
+      <c r="CX16" s="10"/>
+      <c r="CY16" s="23"/>
+      <c r="CZ16" s="23"/>
+      <c r="DA16" s="23"/>
       <c r="DB16" s="23"/>
       <c r="DC16" s="10"/>
-      <c r="DD16" s="10"/>
+      <c r="DD16" s="23"/>
       <c r="DE16" s="10"/>
       <c r="DF16" s="10"/>
       <c r="DG16" s="10"/>
@@ -6833,9 +7038,9 @@
       <c r="DV16" s="10"/>
       <c r="DW16" s="10"/>
       <c r="DX16" s="10"/>
-      <c r="DY16" s="24"/>
+      <c r="DY16" s="10"/>
       <c r="DZ16" s="10"/>
-      <c r="EA16" s="10"/>
+      <c r="EA16" s="24"/>
       <c r="EB16" s="10"/>
       <c r="EC16" s="10"/>
       <c r="ED16" s="10"/>
@@ -6850,13 +7055,20 @@
       <c r="EM16" s="10"/>
       <c r="EN16" s="10"/>
       <c r="EO16" s="10"/>
+      <c r="EP16" s="10"/>
+      <c r="EQ16" s="10"/>
+      <c r="ER16" s="23"/>
+      <c r="ES16" s="10"/>
+      <c r="ET16" s="10"/>
+      <c r="EU16" s="10"/>
+      <c r="EV16" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A7:A16"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="CX5" r:id="rId1" xr:uid="{6592FA46-4216-41E6-9BFC-376DD403D7ED}"/>
+    <hyperlink ref="CZ5" r:id="rId1" xr:uid="{6592FA46-4216-41E6-9BFC-376DD403D7ED}"/>
     <hyperlink ref="CC4" r:id="rId2" xr:uid="{52C90264-B3A6-4214-873C-BB86D485CBFA}"/>
     <hyperlink ref="CB5" r:id="rId3" xr:uid="{7FB6A789-D621-4988-B107-E8BAC64828F6}"/>
     <hyperlink ref="CB4" r:id="rId4" xr:uid="{01F0DA22-AD76-44A4-9D99-DD5EAE634306}"/>
@@ -6895,48 +7107,54 @@
     <hyperlink ref="AF4" r:id="rId37" xr:uid="{043D07EC-33CA-48F9-9214-0ED5BEB776CD}"/>
     <hyperlink ref="AD5" r:id="rId38" xr:uid="{143B8C4A-4E44-4AE6-B837-6E60BB10B7CE}"/>
     <hyperlink ref="AD4" r:id="rId39" xr:uid="{E6789A15-5938-4B34-9060-B643446ED004}"/>
-    <hyperlink ref="DN5" r:id="rId40" xr:uid="{519370B5-9E22-4546-8E09-9C4141372EC4}"/>
-    <hyperlink ref="DK5" r:id="rId41" xr:uid="{0BCBBCDA-D54E-473F-A6FF-214BAF7E0602}"/>
-    <hyperlink ref="CY5" r:id="rId42" xr:uid="{72B74336-2CEF-41FE-9DEA-569F537AAC53}"/>
+    <hyperlink ref="DP5" r:id="rId40" xr:uid="{519370B5-9E22-4546-8E09-9C4141372EC4}"/>
+    <hyperlink ref="DM5" r:id="rId41" xr:uid="{0BCBBCDA-D54E-473F-A6FF-214BAF7E0602}"/>
+    <hyperlink ref="DC5" r:id="rId42" xr:uid="{72B74336-2CEF-41FE-9DEA-569F537AAC53}"/>
     <hyperlink ref="CG5" r:id="rId43" xr:uid="{92CA06A8-10D6-CC41-8669-4699E705FA58}"/>
     <hyperlink ref="CH5:CK5" r:id="rId44" display="http://hl7.org/fhir/us/core/StructureDefinition/us-core-condition-encounter-diagnosis" xr:uid="{9F91280B-E09F-9940-9CC4-44D4A6BECC7B}"/>
     <hyperlink ref="CM5" r:id="rId45" xr:uid="{9E08B7FF-5781-864B-8C4E-B2D12E822AE4}"/>
     <hyperlink ref="CL5" r:id="rId46" xr:uid="{9D824104-EF57-BF43-BAF9-005D49318298}"/>
     <hyperlink ref="CN5:CR5" r:id="rId47" display="http://hl7.org/fhir/us/core/StructureDefinition/us-core-condition-problems-health-concerns" xr:uid="{7357B0DA-F7D4-3846-8F4E-7F1654780E72}"/>
     <hyperlink ref="BO5" r:id="rId48" xr:uid="{CD519393-7745-CD40-976A-BB5E1CCF7CD7}"/>
-    <hyperlink ref="DO5" r:id="rId49" xr:uid="{6F5E54AD-A5E5-314F-862C-49C9A78675A9}"/>
-    <hyperlink ref="DP5" r:id="rId50" xr:uid="{7224C85E-0BF8-424B-B5B2-61993F7E608E}"/>
-    <hyperlink ref="DQ5" r:id="rId51" xr:uid="{722A088B-4E1D-894B-B2FE-467788CD3BCB}"/>
-    <hyperlink ref="DR5" r:id="rId52" xr:uid="{22C91E6F-8D10-9842-8BB7-748A8CCEBE32}"/>
-    <hyperlink ref="DS5" r:id="rId53" xr:uid="{F3D4ED5A-04B2-7B43-B47F-3552A8B0B396}"/>
-    <hyperlink ref="DT5" r:id="rId54" xr:uid="{D1CBDDD6-325F-AF42-A842-7CE4E94A60EE}"/>
-    <hyperlink ref="DU5" r:id="rId55" xr:uid="{08FBAFD1-9D61-044E-BABB-AFDD34782D05}"/>
-    <hyperlink ref="DV5" r:id="rId56" xr:uid="{0BBF327F-B8B8-F640-8E89-8FAE5402534B}"/>
-    <hyperlink ref="DW5" r:id="rId57" xr:uid="{CFBB3623-64B7-3A45-9EF8-53C943C87D44}"/>
-    <hyperlink ref="DX5" r:id="rId58" xr:uid="{1E26B423-EF13-5744-8FB7-F87C92FF385A}"/>
-    <hyperlink ref="DY5" r:id="rId59" xr:uid="{70139C47-100E-DB46-8519-76868848B192}"/>
+    <hyperlink ref="DQ5" r:id="rId49" xr:uid="{6F5E54AD-A5E5-314F-862C-49C9A78675A9}"/>
+    <hyperlink ref="DR5" r:id="rId50" xr:uid="{7224C85E-0BF8-424B-B5B2-61993F7E608E}"/>
+    <hyperlink ref="DS5" r:id="rId51" xr:uid="{722A088B-4E1D-894B-B2FE-467788CD3BCB}"/>
+    <hyperlink ref="DT5" r:id="rId52" xr:uid="{22C91E6F-8D10-9842-8BB7-748A8CCEBE32}"/>
+    <hyperlink ref="DU5" r:id="rId53" xr:uid="{F3D4ED5A-04B2-7B43-B47F-3552A8B0B396}"/>
+    <hyperlink ref="DV5" r:id="rId54" xr:uid="{D1CBDDD6-325F-AF42-A842-7CE4E94A60EE}"/>
+    <hyperlink ref="DW5" r:id="rId55" xr:uid="{08FBAFD1-9D61-044E-BABB-AFDD34782D05}"/>
+    <hyperlink ref="DX5" r:id="rId56" xr:uid="{0BBF327F-B8B8-F640-8E89-8FAE5402534B}"/>
+    <hyperlink ref="DY5" r:id="rId57" xr:uid="{CFBB3623-64B7-3A45-9EF8-53C943C87D44}"/>
+    <hyperlink ref="DZ5" r:id="rId58" xr:uid="{1E26B423-EF13-5744-8FB7-F87C92FF385A}"/>
+    <hyperlink ref="EA5" r:id="rId59" xr:uid="{70139C47-100E-DB46-8519-76868848B192}"/>
     <hyperlink ref="BT5" r:id="rId60" xr:uid="{01EC162A-7861-6C46-B6C6-369B9F1331F8}"/>
     <hyperlink ref="BV5" r:id="rId61" xr:uid="{6D95B09F-5D7E-7344-870D-3090909AAEF4}"/>
-    <hyperlink ref="DZ5" r:id="rId62" xr:uid="{5028E287-1B65-DF4A-8F33-20385BC69AC5}"/>
-    <hyperlink ref="EA5:EC5" r:id="rId63" display="http://hl7.org/fhir/us/core/StructureDefinition/us-core-servicerequest" xr:uid="{E0BF5631-D2C1-4A47-9C6E-09B7D0F51C95}"/>
-    <hyperlink ref="DL5" r:id="rId64" xr:uid="{849A955B-0D4E-8442-8CA3-3E2505A237A3}"/>
-    <hyperlink ref="DM5" r:id="rId65" xr:uid="{B9C03468-74AD-8545-941B-B6346D33A378}"/>
-    <hyperlink ref="ED5" r:id="rId66" xr:uid="{058ADC11-D76F-8A44-8FF2-CF1DD58657F4}"/>
-    <hyperlink ref="ED7" r:id="rId67" xr:uid="{76B4A4C3-F620-294F-B07F-36E44435B509}"/>
-    <hyperlink ref="EE5:EG5" r:id="rId68" display="http://hl7.org/fhir/us/odh/StructureDefinition/odh-UsualWork" xr:uid="{C1DC378C-A920-C94C-86AB-5AD8AFAF335C}"/>
-    <hyperlink ref="EE5" r:id="rId69" xr:uid="{90A04B1B-2387-7145-B4C5-65AEBF36B6BF}"/>
-    <hyperlink ref="EH5" r:id="rId70" xr:uid="{5F45FC77-8D58-F344-8C34-34B11582A41D}"/>
-    <hyperlink ref="EI5" r:id="rId71" xr:uid="{EFDDC6B3-5206-AB4B-8367-206AC1B29EA0}"/>
-    <hyperlink ref="EK5" r:id="rId72" xr:uid="{98BF0F1D-F44E-A544-BD9A-819A1F0775F2}"/>
-    <hyperlink ref="EK4" r:id="rId73" xr:uid="{65C1B558-168A-4F4E-A855-16D87796C211}"/>
-    <hyperlink ref="EO4" r:id="rId74" xr:uid="{EB56323F-1B2E-CA4A-841D-8D20DC90800B}"/>
-    <hyperlink ref="EJ4" r:id="rId75" xr:uid="{B59DC2D6-2E40-7440-8BDB-4E6120670694}"/>
-    <hyperlink ref="EO5" r:id="rId76" xr:uid="{1BB9C402-2A9C-1040-BF9B-0D22FCF407E0}"/>
-    <hyperlink ref="EM5" r:id="rId77" xr:uid="{BE80C563-B20B-0A40-BEBF-347FB731295B}"/>
-    <hyperlink ref="EJ5" r:id="rId78" xr:uid="{43C1F3F8-A3CE-904F-8AA8-D9D9C3DF991D}"/>
-    <hyperlink ref="EL5" r:id="rId79" xr:uid="{CDD43975-5BD5-064D-8BCC-0199351FAE79}"/>
-    <hyperlink ref="EN5" r:id="rId80" xr:uid="{1EC99C06-4DFA-5744-B2FD-EF6D5335B91B}"/>
-    <hyperlink ref="EL7" r:id="rId81" xr:uid="{CDED130F-8B5B-9C48-B37B-54A9359AE8D2}"/>
+    <hyperlink ref="EB5" r:id="rId62" xr:uid="{5028E287-1B65-DF4A-8F33-20385BC69AC5}"/>
+    <hyperlink ref="EC5:EE5" r:id="rId63" display="http://hl7.org/fhir/us/core/StructureDefinition/us-core-servicerequest" xr:uid="{E0BF5631-D2C1-4A47-9C6E-09B7D0F51C95}"/>
+    <hyperlink ref="DN5" r:id="rId64" xr:uid="{849A955B-0D4E-8442-8CA3-3E2505A237A3}"/>
+    <hyperlink ref="DO5" r:id="rId65" xr:uid="{B9C03468-74AD-8545-941B-B6346D33A378}"/>
+    <hyperlink ref="EF5" r:id="rId66" xr:uid="{058ADC11-D76F-8A44-8FF2-CF1DD58657F4}"/>
+    <hyperlink ref="EF7" r:id="rId67" xr:uid="{76B4A4C3-F620-294F-B07F-36E44435B509}"/>
+    <hyperlink ref="EG5:EI5" r:id="rId68" display="http://hl7.org/fhir/us/odh/StructureDefinition/odh-UsualWork" xr:uid="{C1DC378C-A920-C94C-86AB-5AD8AFAF335C}"/>
+    <hyperlink ref="EG5" r:id="rId69" xr:uid="{90A04B1B-2387-7145-B4C5-65AEBF36B6BF}"/>
+    <hyperlink ref="EJ5" r:id="rId70" xr:uid="{5F45FC77-8D58-F344-8C34-34B11582A41D}"/>
+    <hyperlink ref="EK5" r:id="rId71" xr:uid="{EFDDC6B3-5206-AB4B-8367-206AC1B29EA0}"/>
+    <hyperlink ref="EM4" r:id="rId72" xr:uid="{65C1B558-168A-4F4E-A855-16D87796C211}"/>
+    <hyperlink ref="EQ4" r:id="rId73" xr:uid="{EB56323F-1B2E-CA4A-841D-8D20DC90800B}"/>
+    <hyperlink ref="EL4" r:id="rId74" xr:uid="{B59DC2D6-2E40-7440-8BDB-4E6120670694}"/>
+    <hyperlink ref="EL5" r:id="rId75" xr:uid="{43C1F3F8-A3CE-904F-8AA8-D9D9C3DF991D}"/>
+    <hyperlink ref="EN7" r:id="rId76" xr:uid="{CDED130F-8B5B-9C48-B37B-54A9359AE8D2}"/>
+    <hyperlink ref="ES5" r:id="rId77" xr:uid="{55E56568-67ED-4147-A94D-E501A5CF63F1}"/>
+    <hyperlink ref="CY5" r:id="rId78" xr:uid="{B3CB5991-69E9-2D44-BADE-95F36ACDC928}"/>
+    <hyperlink ref="CY4" r:id="rId79" xr:uid="{AB1CE32B-5595-8649-B17D-72F727C03985}"/>
+    <hyperlink ref="CY7" r:id="rId80" xr:uid="{4822A303-D79E-664E-B23D-251E80D0EDEC}"/>
+    <hyperlink ref="DB5" r:id="rId81" xr:uid="{8739BCAA-E0E8-8646-B056-14B0970BBA4C}"/>
+    <hyperlink ref="DA5" r:id="rId82" xr:uid="{945812CB-1FA2-6E4A-B10C-297E0C43CFFB}"/>
+    <hyperlink ref="ER5" r:id="rId83" xr:uid="{DFA51A51-8D0A-3D4E-8185-A052E9A0C1B8}"/>
+    <hyperlink ref="ER4" r:id="rId84" xr:uid="{856C55C7-2427-F745-BFEC-2176C02C221D}"/>
+    <hyperlink ref="ER7" r:id="rId85" xr:uid="{77FCD007-F0EC-B542-8FD7-02865FCA7121}"/>
+    <hyperlink ref="EV5" r:id="rId86" xr:uid="{05F9F0E4-1080-024D-94AF-0F7CD3E27B34}"/>
+    <hyperlink ref="EM5:EQ5" r:id="rId87" display="http://hl7.org/fhir/us/core/StructureDefinition/us-core-observation-pregnancystatus" xr:uid="{297F7906-37EA-C54B-9C2D-B7707EC9223B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -8131,7 +8349,7 @@
       </c>
     </row>
     <row r="6" spans="1:84" ht="32" x14ac:dyDescent="0.2">
-      <c r="A6" s="128"/>
+      <c r="A6" s="129"/>
       <c r="B6" s="103"/>
       <c r="C6" s="104" t="s">
         <v>336</v>
@@ -8235,7 +8453,7 @@
       <c r="CF6" s="107"/>
     </row>
     <row r="7" spans="1:84" ht="32" x14ac:dyDescent="0.2">
-      <c r="A7" s="129"/>
+      <c r="A7" s="130"/>
       <c r="B7" s="103"/>
       <c r="C7" s="108" t="s">
         <v>337</v>
@@ -8273,7 +8491,7 @@
       <c r="CF7" s="111"/>
     </row>
     <row r="8" spans="1:84" ht="32" x14ac:dyDescent="0.2">
-      <c r="A8" s="129"/>
+      <c r="A8" s="130"/>
       <c r="B8" s="103"/>
       <c r="C8" s="108" t="s">
         <v>338</v>
@@ -8305,7 +8523,7 @@
       <c r="CF8" s="111"/>
     </row>
     <row r="9" spans="1:84" ht="32" x14ac:dyDescent="0.2">
-      <c r="A9" s="129"/>
+      <c r="A9" s="130"/>
       <c r="B9" s="103"/>
       <c r="C9" s="108" t="s">
         <v>339</v>
@@ -8334,7 +8552,7 @@
       <c r="CF9" s="111"/>
     </row>
     <row r="10" spans="1:84" ht="48" x14ac:dyDescent="0.2">
-      <c r="A10" s="129"/>
+      <c r="A10" s="130"/>
       <c r="B10" s="103"/>
       <c r="C10" s="108" t="s">
         <v>340</v>
@@ -8363,7 +8581,7 @@
       <c r="CF10" s="111"/>
     </row>
     <row r="11" spans="1:84" ht="48" x14ac:dyDescent="0.2">
-      <c r="A11" s="129"/>
+      <c r="A11" s="130"/>
       <c r="B11" s="103"/>
       <c r="C11" s="108"/>
       <c r="F11" s="2" t="s">
@@ -8387,7 +8605,7 @@
       <c r="CF11" s="111"/>
     </row>
     <row r="12" spans="1:84" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="129"/>
+      <c r="A12" s="130"/>
       <c r="B12" s="103"/>
       <c r="C12" s="108"/>
       <c r="F12" s="2" t="s">
@@ -8411,7 +8629,7 @@
       <c r="CF12" s="111"/>
     </row>
     <row r="13" spans="1:84" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="129"/>
+      <c r="A13" s="130"/>
       <c r="B13" s="103"/>
       <c r="C13" s="108"/>
       <c r="J13" s="97" t="s">
@@ -8429,7 +8647,7 @@
       <c r="CF13" s="111"/>
     </row>
     <row r="14" spans="1:84" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="129"/>
+      <c r="A14" s="130"/>
       <c r="B14" s="103"/>
       <c r="C14" s="108"/>
       <c r="J14" s="97" t="s">
@@ -8447,7 +8665,7 @@
       <c r="CF14" s="111"/>
     </row>
     <row r="15" spans="1:84" ht="33" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="130"/>
+      <c r="A15" s="131"/>
       <c r="B15" s="112"/>
       <c r="C15" s="113"/>
       <c r="D15" s="114"/>

</xml_diff>